<commit_message>
updated file with content
</commit_message>
<xml_diff>
--- a/week-01/Ex2B_data_roundup.xlsx
+++ b/week-01/Ex2B_data_roundup.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nataliamiranda\Documents\DataAnalytics\week-01\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{877F8E2B-C551-42E1-8E6D-89B23659C65C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,104 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
+  <si>
+    <t>Name of data source</t>
+  </si>
+  <si>
+    <t>Type of info (e.g. social media, health, communication, purchases, services)</t>
+  </si>
+  <si>
+    <t>Depth of coverage (i.e. How far back does the data go?)</t>
+  </si>
+  <si>
+    <t>Downloadable?</t>
+  </si>
+  <si>
+    <t>Steps to download</t>
+  </si>
+  <si>
+    <t>Download format (e.g. .csv, .json, .pdf, etc)</t>
+  </si>
+  <si>
+    <t>Additional notes (optional, if you want to jot down any observations)</t>
+  </si>
+  <si>
+    <t>Instagram</t>
+  </si>
+  <si>
+    <t>Social Media</t>
+  </si>
+  <si>
+    <t>Since account creation</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Settings → Accounts Center → Your information and permissions → Download your information</t>
+  </si>
+  <si>
+    <t>.json and HTML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Includes messages, posts, and activity history
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chase Bank </t>
+  </si>
+  <si>
+    <t>Financial</t>
+  </si>
+  <si>
+    <t>Up to 7 years (depending on account)</t>
+  </si>
+  <si>
+    <t>Login → Accounts → Statements &amp; Documents → Download</t>
+  </si>
+  <si>
+    <t>.pdf and .csv</t>
+  </si>
+  <si>
+    <t>.CVS use for data analysis</t>
+  </si>
+  <si>
+    <t>Gmail</t>
+  </si>
+  <si>
+    <t>Communication</t>
+  </si>
+  <si>
+    <t>Google Account → Data &amp; Privacy → Download your data (Google Takeout)</t>
+  </si>
+  <si>
+    <t>MBOX and ZIP</t>
+  </si>
+  <si>
+    <t>MBOX requires a special software to open</t>
+  </si>
+  <si>
+    <t>MyChart</t>
+  </si>
+  <si>
+    <t>Health</t>
+  </si>
+  <si>
+    <t>Varies by provider (On my end my provider is Stanford and I can see all my records since I created the account)</t>
+  </si>
+  <si>
+    <t>Menu → Sharing → Download/Export medical record</t>
+  </si>
+  <si>
+    <t>May include lab results and visit summaries</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -29,12 +131,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,14 +157,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFFFCC"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -330,10 +449,129 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultColWidth="22.36328125" defaultRowHeight="78" customHeight="1" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="16384" width="22.36328125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="78" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="78" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="78" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="78" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="78" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>